<commit_message>
test case document for latest version
test case document for latest version of the application on 10th june 2026
</commit_message>
<xml_diff>
--- a/test case document.xlsx
+++ b/test case document.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="152511" iterateDelta="1E-4"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -226,9 +226,6 @@
     <t>Minimum/maximum field length limits are not enforced, and data type constraints are not validated. Error messages must be added.</t>
   </si>
   <si>
-    <t xml:space="preserve"> Error messages for invalid inputs</t>
-  </si>
-  <si>
     <t>Verify that meaningful error messages are displayed when invalid data is entered.</t>
   </si>
   <si>
@@ -244,9 +241,6 @@
     <t>No error message displayed for invalid inputs when navigating away.</t>
   </si>
   <si>
-    <t>Missing inline error messages for invalid inputs. Error handling must be implemented for all form fields.</t>
-  </si>
-  <si>
     <t>DXF File Import</t>
   </si>
   <si>
@@ -331,9 +325,6 @@
     <t>Application remains fully responsive throughout the processing; no crash or 'Not Responding' state occurs.</t>
   </si>
   <si>
-    <t>Application crashed or entered 'Not Responding' state when opening Drawing Preview or 3D View. Core functionality remained responsive.</t>
-  </si>
-  <si>
     <t>Known limitation: Drawing Preview and 3D View may be unresponsive for very large files. Recommended hardware specs should be documented for end users.</t>
   </si>
   <si>
@@ -602,13 +593,46 @@
   </si>
   <si>
     <t>Audit logs are incomplete. Logging must be added for login events (username and success/failure status) and other key actions.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> Error messages for invalid inputs(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Not mandator</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>y)</t>
+    </r>
+  </si>
+  <si>
+    <t>Application entered 'Not Responding' state when opening Drawing Preview or 3D View. Core functionality remained responsive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing error messages for invalid inputs and empty field. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -629,6 +653,29 @@
       <sz val="11"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="7" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -651,7 +698,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -666,6 +713,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1182,59 +1238,59 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B9" s="3" t="s">
+    <row r="9" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="B9" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>70</v>
+      <c r="J9" s="7" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="D10" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>78</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>17</v>
@@ -1243,27 +1299,27 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>17</v>
@@ -1274,83 +1330,83 @@
     </row>
     <row r="12" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="I12" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>98</v>
-      </c>
       <c r="H13" s="1" t="s">
-        <v>99</v>
+        <v>188</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>21</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="H14" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>17</v>
@@ -1359,30 +1415,30 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="116" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>17</v>
@@ -1391,27 +1447,27 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B16" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H16" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>17</v>
@@ -1422,28 +1478,28 @@
     </row>
     <row r="17" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="E17" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="H17" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>17</v>
@@ -1454,25 +1510,25 @@
     </row>
     <row r="18" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="H18" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>17</v>
@@ -1483,25 +1539,25 @@
     </row>
     <row r="19" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B19" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>17</v>
@@ -1510,27 +1566,27 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B20" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="H20" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>17</v>
@@ -1539,30 +1595,30 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="H21" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>25</v>
@@ -1573,25 +1629,25 @@
     </row>
     <row r="22" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="H22" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>17</v>
@@ -1600,30 +1656,30 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="116" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>27</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>25</v>
@@ -1637,25 +1693,25 @@
         <v>28</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="F24" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="H24" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>174</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>17</v>
@@ -1666,25 +1722,25 @@
     </row>
     <row r="25" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="H25" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>17</v>
@@ -1693,36 +1749,36 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="G26" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="H26" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>21</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>